<commit_message>
Update exam portal data and add exam results
</commit_message>
<xml_diff>
--- a/data/exam_portal.xlsx
+++ b/data/exam_portal.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Users" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exams" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Users" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Questions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Exams" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Results" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -495,6 +495,33 @@
         </is>
       </c>
       <c r="E3" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>0c8c4361-a819-41b7-b19e-b4ceba1719b6</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Karan</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>kt241072@gmail.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>scrypt:32768:8:1$Ywq9nqOMdkZw9iVx$116c9acc660aa9334ae09775211ab01c777ff31b3eb67e89731ec0547cd58d7b5e2d0190f92898c1b932252bef5c56a0e3fea052a3357deeac22b96e5a45b52e</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
         <is>
           <t>student</t>
         </is>

</xml_diff>